<commit_message>
Fix lab unit display
</commit_message>
<xml_diff>
--- a/templates/future-case-template.xlsx
+++ b/templates/future-case-template.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Case" sheetId="1" r:id="R444fd539a1a44bf5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Medications" sheetId="2" r:id="R3b2e147d8bac4e7c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Previous Meds" sheetId="3" r:id="R5d848b0003e24320"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Answer" sheetId="4" r:id="R5f3a2efe4a3e42b6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="References" sheetId="5" r:id="Rea3616844c3642b5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instructions" sheetId="6" r:id="Re5647dfde462422c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Case" sheetId="1" r:id="Rae5b99caf0434271"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Medications" sheetId="2" r:id="R9b05aeaddcda4618"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Previous Meds" sheetId="3" r:id="R0454e70a70fe4917"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Answer" sheetId="4" r:id="R9a592cfc33ca4212"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="References" sheetId="5" r:id="Reded9e7f0c0f4d59"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instructions" sheetId="6" r:id="R87b45bce40c047bf"/>
   </x:sheets>
 </x:workbook>
 </file>

</xml_diff>